<commit_message>
docs: align guides, specs and registry with Decisions D1–D16 and review fixes
</commit_message>
<xml_diff>
--- a/apps/docs/public/samples/opening-balances-example.xlsx
+++ b/apps/docs/public/samples/opening-balances-example.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>Template version</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>GST supply class: taxable, exempt, nil, nonGst, notASupply.</t>
+  </si>
+  <si>
+    <t>Tax code: taxable items use your organization's GST rate codes (GST5, GST12, GST18, GST28, GST40); check which rates are effective in Items.</t>
   </si>
   <si>
     <t>Opening date</t>
@@ -356,7 +359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -390,6 +393,11 @@
     <row r="6">
       <c r="A6" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -404,7 +412,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -424,24 +432,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -456,56 +464,56 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
         <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -520,30 +528,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -561,18 +569,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <v>20000</v>
@@ -580,7 +588,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>8000</v>
@@ -588,7 +596,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -596,7 +604,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5">
         <v>23000</v>
@@ -614,45 +622,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G2">
         <v>10000</v>
@@ -660,42 +668,42 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G4">
         <v>5000</v>

</xml_diff>